<commit_message>
Docs: 13-sheet company book (payroll & pension added) + full book PDF export
</commit_message>
<xml_diff>
--- a/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
+++ b/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Customers" sheetId="10" r:id="rId10"/>
     <sheet name="Money In" sheetId="11" r:id="rId11"/>
     <sheet name="Money Out" sheetId="12" r:id="rId12"/>
+    <sheet name="Payroll &amp; Pension" sheetId="13" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company Forecast'!$A$1:$F$1</definedName>
@@ -29,6 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Money In'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Money Out'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Payments!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Payroll &amp; Pension'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Quotes!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Suppliers!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Tax!$A$1:$J$1</definedName>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="286">
   <si>
     <t>Priority</t>
   </si>
@@ -380,6 +382,12 @@
     <t>quote; est SME</t>
   </si>
   <si>
+    <t>Payroll / pension provider</t>
+  </si>
+  <si>
+    <t>Xero/PayeZone or free; when staff</t>
+  </si>
+  <si>
     <t>ISO 27001 (later)</t>
   </si>
   <si>
@@ -716,6 +724,27 @@
     <t>book now</t>
   </si>
   <si>
+    <t>Pension provider (future)</t>
+  </si>
+  <si>
+    <t>NEST/The People's Pension</t>
+  </si>
+  <si>
+    <t>auto-enrolment</t>
+  </si>
+  <si>
+    <t>when staff hired</t>
+  </si>
+  <si>
+    <t>Payroll provider (future)</t>
+  </si>
+  <si>
+    <t>PayeZone/Xero</t>
+  </si>
+  <si>
+    <t>PAYE/RTI filing</t>
+  </si>
+  <si>
     <t>UKAS body (future)</t>
   </si>
   <si>
@@ -828,6 +857,48 @@
   </si>
   <si>
     <t>Receipt</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Gross £</t>
+  </si>
+  <si>
+    <t>PAYE/NI £</t>
+  </si>
+  <si>
+    <t>Net pay £</t>
+  </si>
+  <si>
+    <t>Pension EE £</t>
+  </si>
+  <si>
+    <t>Pension ER £</t>
+  </si>
+  <si>
+    <t>Pension total £</t>
+  </si>
+  <si>
+    <t>RTI filed</t>
+  </si>
+  <si>
+    <t>Darren Birch (Director)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Hire 1 (future)</t>
+  </si>
+  <si>
+    <t>TOTALS</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>Auto-enrolment: ER min 3% of qualifying earnings, EE 5%; register pension scheme + join RTI before hiring. Directors can be opted-in or excluded per HMRC rules.</t>
   </si>
 </sst>
 </file>
@@ -862,7 +933,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -899,6 +970,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F4C5C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -927,7 +1004,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -945,6 +1022,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1820,10 +1901,10 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>82</v>
@@ -1835,7 +1916,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>89</v>
@@ -1843,119 +1924,119 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="B3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F3" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B4" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C4" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E4" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F4" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F5" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>257</v>
+      </c>
+      <c r="B6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D6" t="s">
         <v>248</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>249</v>
       </c>
-      <c r="C6" t="s">
-        <v>238</v>
-      </c>
-      <c r="D6" t="s">
-        <v>239</v>
-      </c>
-      <c r="E6" t="s">
-        <v>240</v>
-      </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="B7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C7" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="D7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="G7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -1980,28 +2061,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2123,19 +2204,19 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -2144,7 +2225,7 @@
         <v>87</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2245,6 +2326,790 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="34.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" s="4">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C18" s="4">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" s="4">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C21" s="4">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" s="4">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C23" s="4">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C24" s="4">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C25" s="4">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C26" s="4">
+        <f>SUM(C2:C24)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="4">
+        <f>SUM(D2:D24)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <f>SUM(E2:E24)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="4">
+        <f>SUM(F2:F24)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <f>SUM(G2:G24)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="4">
+        <f>SUM(H2:H24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2417,7 +3282,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -2529,10 +3394,10 @@
         <v>113</v>
       </c>
       <c r="B8" s="4">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="C8" s="4">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>114</v>
@@ -2543,27 +3408,41 @@
         <v>115</v>
       </c>
       <c r="B9" s="4">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="C9" s="4">
-        <v>485</v>
+        <v>5000</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>485</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="8">
         <v>2240</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C11" s="8">
         <v>102</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>118</v>
+      <c r="D11" s="8" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2586,19 +3465,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>89</v>
@@ -2606,7 +3485,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B2" s="4">
         <v>0</v>
@@ -2621,12 +3500,12 @@
         <v>-10.5</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B3" s="4">
         <v>0</v>
@@ -2641,12 +3520,12 @@
         <v>-21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B4" s="4">
         <v>0</v>
@@ -2661,12 +3540,12 @@
         <v>-31.56</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B5" s="4">
         <v>5000</v>
@@ -2681,12 +3560,12 @@
         <v>4957.94</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B6" s="4">
         <v>6500</v>
@@ -2701,12 +3580,12 @@
         <v>11447.44</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B7" s="4">
         <v>8000</v>
@@ -2721,12 +3600,12 @@
         <v>19436.94</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B8" s="4">
         <v>9500</v>
@@ -2741,12 +3620,12 @@
         <v>28926.44</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B9" s="4">
         <v>11000</v>
@@ -2761,12 +3640,12 @@
         <v>39915.94</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B10" s="4">
         <v>12500</v>
@@ -2781,12 +3660,12 @@
         <v>52405.44</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B11" s="4">
         <v>14000</v>
@@ -2801,12 +3680,12 @@
         <v>66394.94</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B12" s="4">
         <v>15500</v>
@@ -2821,12 +3700,12 @@
         <v>81884.44</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" s="4">
         <v>17000</v>
@@ -2841,7 +3720,7 @@
         <v>98873.94</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2887,39 +3766,39 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -2931,12 +3810,12 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2948,29 +3827,29 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>150</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2982,12 +3861,12 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -2999,12 +3878,12 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -3016,12 +3895,12 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -3033,12 +3912,12 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -3050,12 +3929,12 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -3067,12 +3946,12 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -3084,7 +3963,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3108,34 +3987,34 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>87</v>
@@ -3143,7 +4022,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -3155,12 +4034,12 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -3172,29 +4051,29 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
         <v>163</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -3206,12 +4085,12 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -3223,12 +4102,12 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -3240,12 +4119,12 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -3257,12 +4136,12 @@
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -3274,12 +4153,12 @@
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -3291,12 +4170,12 @@
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -3308,12 +4187,12 @@
         <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -3325,12 +4204,12 @@
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -3342,7 +4221,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -3368,39 +4247,39 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3411,7 +4290,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -3422,7 +4301,7 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -3433,7 +4312,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -3444,7 +4323,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -3455,7 +4334,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -3466,7 +4345,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -3477,7 +4356,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -3488,7 +4367,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -3499,7 +4378,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -3510,7 +4389,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -3521,7 +4400,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -3553,31 +4432,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -3585,7 +4464,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -3597,12 +4476,12 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3614,29 +4493,29 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
         <v>201</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3648,12 +4527,12 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -3665,7 +4544,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3676,7 +4555,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -3689,22 +4568,22 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>89</v>
@@ -3712,41 +4591,41 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E3" t="s">
         <v>215</v>
-      </c>
-      <c r="C3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E3" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E4" t="s">
         <v>50</v>
@@ -3754,16 +4633,16 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E5" t="s">
         <v>50</v>
       </c>
       <c r="G5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3771,41 +4650,75 @@
         <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E6" t="s">
         <v>50</v>
       </c>
       <c r="G6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>225</v>
+        <v>227</v>
+      </c>
+      <c r="B7" t="s">
+        <v>228</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>229</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>215</v>
       </c>
       <c r="G7" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>227</v>
+        <v>231</v>
+      </c>
+      <c r="B8" t="s">
+        <v>232</v>
       </c>
       <c r="C8" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E8" t="s">
+        <v>215</v>
+      </c>
+      <c r="G8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" t="s">
         <v>50</v>
       </c>
-      <c r="G8" t="s">
-        <v>229</v>
+      <c r="G9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C10" t="s">
+        <v>237</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docs: 13-sheet company book + full PDF (PR #30)
* Docs: AEGIS security fixes changelog + operating costs + cost forecast spreadsheet

* Docs: Monday NHS readiness summary

* Docs: trademark applications draft + DTAC submission answers + compliance tracker

* Docs: series application checklist + compliance tracker template + NHS trademark/IP research

* Docs: tracker with IPO-number sheet + NHS background-IP contract clause draft

* Docs: 12-sheet company book (tracker+forecast+quotes+invoices+tax+suppliers+customers+money) + tracker PDF + IP clause solicitor notes

* Docs: 13-sheet company book (payroll & pension added) + full book PDF export

---------

Co-authored-by: Higgsfield Agent <agent@higgsfield.ai>
</commit_message>
<xml_diff>
--- a/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
+++ b/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Customers" sheetId="10" r:id="rId10"/>
     <sheet name="Money In" sheetId="11" r:id="rId11"/>
     <sheet name="Money Out" sheetId="12" r:id="rId12"/>
+    <sheet name="Payroll &amp; Pension" sheetId="13" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Company Forecast'!$A$1:$F$1</definedName>
@@ -29,6 +30,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Money In'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Money Out'!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Payments!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Payroll &amp; Pension'!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Quotes!$A$1:$J$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Suppliers!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Tax!$A$1:$J$1</definedName>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="286">
   <si>
     <t>Priority</t>
   </si>
@@ -380,6 +382,12 @@
     <t>quote; est SME</t>
   </si>
   <si>
+    <t>Payroll / pension provider</t>
+  </si>
+  <si>
+    <t>Xero/PayeZone or free; when staff</t>
+  </si>
+  <si>
     <t>ISO 27001 (later)</t>
   </si>
   <si>
@@ -716,6 +724,27 @@
     <t>book now</t>
   </si>
   <si>
+    <t>Pension provider (future)</t>
+  </si>
+  <si>
+    <t>NEST/The People's Pension</t>
+  </si>
+  <si>
+    <t>auto-enrolment</t>
+  </si>
+  <si>
+    <t>when staff hired</t>
+  </si>
+  <si>
+    <t>Payroll provider (future)</t>
+  </si>
+  <si>
+    <t>PayeZone/Xero</t>
+  </si>
+  <si>
+    <t>PAYE/RTI filing</t>
+  </si>
+  <si>
     <t>UKAS body (future)</t>
   </si>
   <si>
@@ -828,6 +857,48 @@
   </si>
   <si>
     <t>Receipt</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>Gross £</t>
+  </si>
+  <si>
+    <t>PAYE/NI £</t>
+  </si>
+  <si>
+    <t>Net pay £</t>
+  </si>
+  <si>
+    <t>Pension EE £</t>
+  </si>
+  <si>
+    <t>Pension ER £</t>
+  </si>
+  <si>
+    <t>Pension total £</t>
+  </si>
+  <si>
+    <t>RTI filed</t>
+  </si>
+  <si>
+    <t>Darren Birch (Director)</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Hire 1 (future)</t>
+  </si>
+  <si>
+    <t>TOTALS</t>
+  </si>
+  <si>
+    <t>NOTES</t>
+  </si>
+  <si>
+    <t>Auto-enrolment: ER min 3% of qualifying earnings, EE 5%; register pension scheme + join RTI before hiring. Directors can be opted-in or excluded per HMRC rules.</t>
   </si>
 </sst>
 </file>
@@ -862,7 +933,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -899,6 +970,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0F4C5C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -927,7 +1004,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -945,6 +1022,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1820,10 +1901,10 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>82</v>
@@ -1835,7 +1916,7 @@
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>89</v>
@@ -1843,119 +1924,119 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C2" t="s">
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="F2" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="B3" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="C3" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D3" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E3" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F3" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="B4" t="s">
-        <v>243</v>
+        <v>252</v>
       </c>
       <c r="C4" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D4" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E4" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F4" t="s">
-        <v>244</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>245</v>
+        <v>254</v>
       </c>
       <c r="B5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="C5" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
       <c r="D5" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="E5" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F5" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
+        <v>257</v>
+      </c>
+      <c r="B6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D6" t="s">
         <v>248</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>249</v>
       </c>
-      <c r="C6" t="s">
-        <v>238</v>
-      </c>
-      <c r="D6" t="s">
-        <v>239</v>
-      </c>
-      <c r="E6" t="s">
-        <v>240</v>
-      </c>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="B7" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C7" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="D7" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="G7" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -1980,28 +2061,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2123,19 +2204,19 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -2144,7 +2225,7 @@
         <v>87</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -2245,6 +2326,790 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="34.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C5" s="4">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C7" s="4">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C8" s="4">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4">
+        <v>0</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C9" s="4">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4">
+        <v>0</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0</v>
+      </c>
+      <c r="H9" s="4">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C10" s="4">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C12" s="4">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>0</v>
+      </c>
+      <c r="E12" s="4">
+        <v>0</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0</v>
+      </c>
+      <c r="G12" s="4">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C13" s="4">
+        <v>0</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4">
+        <v>0</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C14" s="4">
+        <v>0</v>
+      </c>
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+      <c r="G14" s="4">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C15" s="4">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>0</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+      <c r="G16" s="4">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" s="4">
+        <v>0</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0</v>
+      </c>
+      <c r="G17" s="4">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C18" s="4">
+        <v>0</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C20" s="4">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0</v>
+      </c>
+      <c r="E20" s="4">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C21" s="4">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C22" s="4">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C23" s="4">
+        <v>0</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4">
+        <v>0</v>
+      </c>
+      <c r="G23" s="4">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4">
+        <v>0</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="C24" s="4">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0</v>
+      </c>
+      <c r="E24" s="4">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C25" s="4">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C26" s="4">
+        <f>SUM(C2:C24)</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="4">
+        <f>SUM(D2:D24)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="4">
+        <f>SUM(E2:E24)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="4">
+        <f>SUM(F2:F24)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="4">
+        <f>SUM(G2:G24)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="4">
+        <f>SUM(H2:H24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2417,7 +3282,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -2529,10 +3394,10 @@
         <v>113</v>
       </c>
       <c r="B8" s="4">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="C8" s="4">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>114</v>
@@ -2543,27 +3408,41 @@
         <v>115</v>
       </c>
       <c r="B9" s="4">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="C9" s="4">
-        <v>485</v>
+        <v>5000</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="4">
+        <v>0</v>
+      </c>
+      <c r="C10" s="4">
+        <v>485</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="8">
         <v>2240</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C11" s="8">
         <v>102</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>118</v>
+      <c r="D11" s="8" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2586,19 +3465,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>89</v>
@@ -2606,7 +3485,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B2" s="4">
         <v>0</v>
@@ -2621,12 +3500,12 @@
         <v>-10.5</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B3" s="4">
         <v>0</v>
@@ -2641,12 +3520,12 @@
         <v>-21</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B4" s="4">
         <v>0</v>
@@ -2661,12 +3540,12 @@
         <v>-31.56</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B5" s="4">
         <v>5000</v>
@@ -2681,12 +3560,12 @@
         <v>4957.94</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B6" s="4">
         <v>6500</v>
@@ -2701,12 +3580,12 @@
         <v>11447.44</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B7" s="4">
         <v>8000</v>
@@ -2721,12 +3600,12 @@
         <v>19436.94</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B8" s="4">
         <v>9500</v>
@@ -2741,12 +3620,12 @@
         <v>28926.44</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B9" s="4">
         <v>11000</v>
@@ -2761,12 +3640,12 @@
         <v>39915.94</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B10" s="4">
         <v>12500</v>
@@ -2781,12 +3660,12 @@
         <v>52405.44</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B11" s="4">
         <v>14000</v>
@@ -2801,12 +3680,12 @@
         <v>66394.94</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B12" s="4">
         <v>15500</v>
@@ -2821,12 +3700,12 @@
         <v>81884.44</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B13" s="4">
         <v>17000</v>
@@ -2841,7 +3720,7 @@
         <v>98873.94</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2887,39 +3766,39 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -2931,12 +3810,12 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2948,29 +3827,29 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4" t="s">
         <v>150</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -2982,12 +3861,12 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -2999,12 +3878,12 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -3016,12 +3895,12 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -3033,12 +3912,12 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -3050,12 +3929,12 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -3067,12 +3946,12 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -3084,7 +3963,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3108,34 +3987,34 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>87</v>
@@ -3143,7 +4022,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -3155,12 +4034,12 @@
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -3172,29 +4051,29 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
         <v>163</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -3206,12 +4085,12 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -3223,12 +4102,12 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -3240,12 +4119,12 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -3257,12 +4136,12 @@
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -3274,12 +4153,12 @@
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -3291,12 +4170,12 @@
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -3308,12 +4187,12 @@
         <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -3325,12 +4204,12 @@
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -3342,7 +4221,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -3368,39 +4247,39 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -3411,7 +4290,7 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -3422,7 +4301,7 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -3433,7 +4312,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -3444,7 +4323,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -3455,7 +4334,7 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -3466,7 +4345,7 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -3477,7 +4356,7 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -3488,7 +4367,7 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -3499,7 +4378,7 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -3510,7 +4389,7 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -3521,7 +4400,7 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -3553,31 +4432,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -3585,7 +4464,7 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -3597,12 +4476,12 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3614,29 +4493,29 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
         <v>201</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3648,12 +4527,12 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -3665,7 +4544,7 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3676,7 +4555,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -3689,22 +4568,22 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>89</v>
@@ -3712,41 +4591,41 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E3" t="s">
         <v>215</v>
-      </c>
-      <c r="C3" t="s">
-        <v>216</v>
-      </c>
-      <c r="E3" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E4" t="s">
         <v>50</v>
@@ -3754,16 +4633,16 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E5" t="s">
         <v>50</v>
       </c>
       <c r="G5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3771,41 +4650,75 @@
         <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E6" t="s">
         <v>50</v>
       </c>
       <c r="G6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>225</v>
+        <v>227</v>
+      </c>
+      <c r="B7" t="s">
+        <v>228</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>229</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>215</v>
       </c>
       <c r="G7" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>227</v>
+        <v>231</v>
+      </c>
+      <c r="B8" t="s">
+        <v>232</v>
       </c>
       <c r="C8" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="E8" t="s">
+        <v>215</v>
+      </c>
+      <c r="G8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" t="s">
         <v>50</v>
       </c>
-      <c r="G8" t="s">
-        <v>229</v>
+      <c r="G9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>236</v>
+      </c>
+      <c r="C10" t="s">
+        <v>237</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Docs: add Domains register sheet (RDAP verified) to company book + PDF
</commit_message>
<xml_diff>
--- a/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
+++ b/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Money In" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Money Out" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Payroll &amp; Pension" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Domains" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +45,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -111,6 +116,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1402,7 +1408,6 @@
           <t>thread 1a043c35ca7bd141</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1435,7 +1440,6 @@
           <t>1a04915860b3a595</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1468,7 +1472,6 @@
           <t>1a04917551880979</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1501,7 +1504,6 @@
           <t>1a049164d596c4c4</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1534,7 +1536,6 @@
           <t>1a04916710805eaa</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1557,8 +1558,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Stripe connected</t>
@@ -1632,172 +1631,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1866,172 +1793,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3119,6 +2974,369 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Registrar</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Expires</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status / verdict</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>zeusaiintelligence.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2027-08-07</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>YOURS (verified RDAP)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ZEUS AI assistant site</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>auto-renew ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>apiaegissecurity.tech</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Porkbun LLC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2027-07-27</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>YOURS (verified RDAP) - locked</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>AEGIS API (droplet)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>auto-renew ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>zeusintelligence.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2019-09-17</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>URGENT - expires in &lt;3 weeks</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>brand-family domain</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CHECK GoDaddy account; renew if yours</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>zeus-ai.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2024-05-26</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2027-05-26</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRM - matches ZEUS brand</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>confirm ownership with Darren</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>jdbsales.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRM - matches JDB Sales</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>confirm ownership with Darren</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>zeusai.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2016-03-12</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2027-03-12</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>likely NOT ours (old)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aegis-ai.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gname 478 Inc</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-12-28</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>likely NOT ours</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>aegissecurity.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>eNom LLC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1999-01-23</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2027-01-23</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>likely NOT ours (1999)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Source: RDAP registry data 29 Aug 2026 (Verisign / rdap.org). Verify against IONOS + Porkbun + GoDaddy accounts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3208,8 +3426,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3218,8 +3434,6 @@
       <c r="G2" t="n">
         <v>445</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>File e-TM3</t>
@@ -3242,8 +3456,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3252,8 +3464,6 @@
       <c r="G3" t="n">
         <v>445</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Separate application</t>
@@ -3276,8 +3486,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3286,8 +3494,6 @@
       <c r="G4" t="n">
         <v>505</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Series app</t>
@@ -3310,8 +3516,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3320,8 +3524,6 @@
       <c r="G5" t="n">
         <v>445</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Consider per contract</t>
@@ -4017,9 +4219,6 @@
           <t>Q-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -4034,8 +4233,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4043,9 +4240,6 @@
           <t>Q-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -4060,8 +4254,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4069,9 +4261,6 @@
           <t>Q-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -4086,8 +4275,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4095,9 +4282,6 @@
           <t>Q-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -4112,8 +4296,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4121,9 +4303,6 @@
           <t>Q-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -4138,8 +4317,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4147,9 +4324,6 @@
           <t>Q-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -4164,8 +4338,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4173,9 +4345,6 @@
           <t>Q-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0</v>
       </c>
@@ -4190,8 +4359,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4199,9 +4366,6 @@
           <t>Q-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -4216,8 +4380,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4225,9 +4387,6 @@
           <t>Q-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0</v>
       </c>
@@ -4242,8 +4401,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4251,9 +4408,6 @@
           <t>Q-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -4268,8 +4422,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4361,10 +4513,6 @@
           <t>INV-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>0</v>
       </c>
@@ -4379,8 +4527,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4388,10 +4534,6 @@
           <t>INV-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>0</v>
       </c>
@@ -4406,8 +4548,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4415,10 +4555,6 @@
           <t>INV-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>0</v>
       </c>
@@ -4433,8 +4569,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4442,10 +4576,6 @@
           <t>INV-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>0</v>
       </c>
@@ -4460,8 +4590,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4469,10 +4597,6 @@
           <t>INV-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>0</v>
       </c>
@@ -4487,8 +4611,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4496,10 +4618,6 @@
           <t>INV-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>0</v>
       </c>
@@ -4514,8 +4632,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4523,10 +4639,6 @@
           <t>INV-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>0</v>
       </c>
@@ -4541,8 +4653,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4550,10 +4660,6 @@
           <t>INV-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>0</v>
       </c>
@@ -4568,8 +4674,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4577,10 +4681,6 @@
           <t>INV-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
         <v>0</v>
       </c>
@@ -4595,8 +4695,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4604,10 +4702,6 @@
           <t>INV-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
         <v>0</v>
       </c>
@@ -4622,8 +4716,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4631,10 +4723,6 @@
           <t>INV-0011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
         <v>0</v>
       </c>
@@ -4649,8 +4737,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4658,10 +4744,6 @@
           <t>INV-0012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
         <v>0</v>
       </c>
@@ -4676,8 +4758,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4763,19 +4843,12 @@
           <t>PAY-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4783,19 +4856,12 @@
           <t>PAY-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4803,19 +4869,12 @@
           <t>PAY-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4823,19 +4882,12 @@
           <t>PAY-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4843,19 +4895,12 @@
           <t>PAY-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4863,19 +4908,12 @@
           <t>PAY-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4883,19 +4921,12 @@
           <t>PAY-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4903,19 +4934,12 @@
           <t>PAY-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4923,19 +4947,12 @@
           <t>PAY-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4943,19 +4960,12 @@
           <t>PAY-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4963,19 +4973,12 @@
           <t>PAY-0011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4983,19 +4986,12 @@
           <t>PAY-0012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5081,9 +5077,6 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -5093,8 +5086,6 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5107,9 +5098,6 @@
           <t>Q2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -5119,8 +5107,6 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5133,9 +5119,6 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -5145,8 +5128,6 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5159,9 +5140,6 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -5171,8 +5149,6 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5185,9 +5161,6 @@
           <t>Year-end CT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -5197,8 +5170,6 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5281,14 +5252,11 @@
           <t>AEGIS hosting</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5306,14 +5274,11 @@
           <t>S3 backups</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5331,14 +5296,11 @@
           <t>DNS/tunnel</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5346,19 +5308,16 @@
           <t>Registrar</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>domains</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>renew before expiry</t>
@@ -5371,19 +5330,16 @@
           <t>IASME</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Cyber Essentials cert</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>book now</t>
@@ -5406,13 +5362,11 @@
           <t>auto-enrolment</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>when staff hired</t>
@@ -5435,13 +5389,11 @@
           <t>PAYE/RTI filing</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>when staff hired</t>
@@ -5454,19 +5406,16 @@
           <t>UKAS body (future)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>ISO 27001</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>post-contract</t>
@@ -5479,19 +5428,16 @@
           <t>Insurer (future)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Cyber/PI</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>get quotes</t>

</xml_diff>

<commit_message>
Docs: Domains register + company book PDF v3 (PR #33)
* Docs: AEGIS security fixes changelog + operating costs + cost forecast spreadsheet

* Docs: Monday NHS readiness summary

* Docs: trademark applications draft + DTAC submission answers + compliance tracker

* Docs: series application checklist + compliance tracker template + NHS trademark/IP research

* Docs: tracker with IPO-number sheet + NHS background-IP contract clause draft

* Docs: 12-sheet company book (tracker+forecast+quotes+invoices+tax+suppliers+customers+money) + tracker PDF + IP clause solicitor notes

* Docs: 13-sheet company book (payroll & pension added) + full book PDF export

* Fix: rebuild company book with max-compatibility xlsx (opens in all viewers)

* Docs: add Domains register sheet (RDAP verified) to company book + PDF

---------

Co-authored-by: Higgsfield Agent <agent@higgsfield.ai>
</commit_message>
<xml_diff>
--- a/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
+++ b/docs/security/ZEUS-AEGIS-COMPANY-BOOK.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Money In" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Money Out" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Payroll &amp; Pension" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Domains" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,6 +45,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -111,6 +116,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1402,7 +1408,6 @@
           <t>thread 1a043c35ca7bd141</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1435,7 +1440,6 @@
           <t>1a04915860b3a595</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1468,7 +1472,6 @@
           <t>1a04917551880979</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1501,7 +1504,6 @@
           <t>1a049164d596c4c4</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1534,7 +1536,6 @@
           <t>1a04916710805eaa</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1557,8 +1558,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>Stripe connected</t>
@@ -1632,172 +1631,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1866,172 +1793,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3119,6 +2974,369 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Registrar</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Expires</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status / verdict</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Used for</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>zeusaiintelligence.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IONOS SE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2027-08-07</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>YOURS (verified RDAP)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ZEUS AI assistant site</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>auto-renew ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>apiaegissecurity.tech</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Porkbun LLC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2027-07-27</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>YOURS (verified RDAP) - locked</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>AEGIS API (droplet)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>auto-renew ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>zeusintelligence.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2019-09-17</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>URGENT - expires in &lt;3 weeks</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>brand-family domain</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CHECK GoDaddy account; renew if yours</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>zeus-ai.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2024-05-26</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2027-05-26</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRM - matches ZEUS brand</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>confirm ownership with Darren</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>jdbsales.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2027-07-01</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>CONFIRM - matches JDB Sales</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>confirm ownership with Darren</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>zeusai.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GoDaddy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2016-03-12</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2027-03-12</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>likely NOT ours (old)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>aegis-ai.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gname 478 Inc</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-12-28</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>likely NOT ours</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>aegissecurity.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>eNom LLC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1999-01-23</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2027-01-23</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>likely NOT ours (1999)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ignore unless confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Source: RDAP registry data 29 Aug 2026 (Verisign / rdap.org). Verify against IONOS + Porkbun + GoDaddy accounts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3208,8 +3426,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3218,8 +3434,6 @@
       <c r="G2" t="n">
         <v>445</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>File e-TM3</t>
@@ -3242,8 +3456,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3252,8 +3464,6 @@
       <c r="G3" t="n">
         <v>445</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Separate application</t>
@@ -3276,8 +3486,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3286,8 +3494,6 @@
       <c r="G4" t="n">
         <v>505</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Series app</t>
@@ -3310,8 +3516,6 @@
           <t>9, 36, 42, 44, 45</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>AWAITING NUMBERS</t>
@@ -3320,8 +3524,6 @@
       <c r="G5" t="n">
         <v>445</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Consider per contract</t>
@@ -4017,9 +4219,6 @@
           <t>Q-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -4034,8 +4233,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4043,9 +4240,6 @@
           <t>Q-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -4060,8 +4254,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4069,9 +4261,6 @@
           <t>Q-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -4086,8 +4275,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4095,9 +4282,6 @@
           <t>Q-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -4112,8 +4296,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4121,9 +4303,6 @@
           <t>Q-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -4138,8 +4317,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4147,9 +4324,6 @@
           <t>Q-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -4164,8 +4338,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4173,9 +4345,6 @@
           <t>Q-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0</v>
       </c>
@@ -4190,8 +4359,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4199,9 +4366,6 @@
           <t>Q-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -4216,8 +4380,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4225,9 +4387,6 @@
           <t>Q-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0</v>
       </c>
@@ -4242,8 +4401,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4251,9 +4408,6 @@
           <t>Q-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -4268,8 +4422,6 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4361,10 +4513,6 @@
           <t>INV-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
         <v>0</v>
       </c>
@@ -4379,8 +4527,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4388,10 +4534,6 @@
           <t>INV-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>0</v>
       </c>
@@ -4406,8 +4548,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4415,10 +4555,6 @@
           <t>INV-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>0</v>
       </c>
@@ -4433,8 +4569,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4442,10 +4576,6 @@
           <t>INV-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>0</v>
       </c>
@@ -4460,8 +4590,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4469,10 +4597,6 @@
           <t>INV-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>0</v>
       </c>
@@ -4487,8 +4611,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4496,10 +4618,6 @@
           <t>INV-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
         <v>0</v>
       </c>
@@ -4514,8 +4632,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4523,10 +4639,6 @@
           <t>INV-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
         <v>0</v>
       </c>
@@ -4541,8 +4653,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4550,10 +4660,6 @@
           <t>INV-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>0</v>
       </c>
@@ -4568,8 +4674,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4577,10 +4681,6 @@
           <t>INV-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
         <v>0</v>
       </c>
@@ -4595,8 +4695,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4604,10 +4702,6 @@
           <t>INV-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
         <v>0</v>
       </c>
@@ -4622,8 +4716,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4631,10 +4723,6 @@
           <t>INV-0011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
         <v>0</v>
       </c>
@@ -4649,8 +4737,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4658,10 +4744,6 @@
           <t>INV-0012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
         <v>0</v>
       </c>
@@ -4676,8 +4758,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4763,19 +4843,12 @@
           <t>PAY-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4783,19 +4856,12 @@
           <t>PAY-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4803,19 +4869,12 @@
           <t>PAY-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4823,19 +4882,12 @@
           <t>PAY-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4843,19 +4895,12 @@
           <t>PAY-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4863,19 +4908,12 @@
           <t>PAY-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4883,19 +4921,12 @@
           <t>PAY-0007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4903,19 +4934,12 @@
           <t>PAY-0008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4923,19 +4947,12 @@
           <t>PAY-0009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4943,19 +4960,12 @@
           <t>PAY-0010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4963,19 +4973,12 @@
           <t>PAY-0011</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4983,19 +4986,12 @@
           <t>PAY-0012</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5081,9 +5077,6 @@
           <t>Q1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -5093,8 +5086,6 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5107,9 +5098,6 @@
           <t>Q2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -5119,8 +5107,6 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5133,9 +5119,6 @@
           <t>Q3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -5145,8 +5128,6 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5159,9 +5140,6 @@
           <t>Q4</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -5171,8 +5149,6 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5185,9 +5161,6 @@
           <t>Year-end CT</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -5197,8 +5170,6 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>Not due</t>
@@ -5281,14 +5252,11 @@
           <t>AEGIS hosting</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5306,14 +5274,11 @@
           <t>S3 backups</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5331,14 +5296,11 @@
           <t>DNS/tunnel</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5346,19 +5308,16 @@
           <t>Registrar</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>domains</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>renew before expiry</t>
@@ -5371,19 +5330,16 @@
           <t>IASME</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Cyber Essentials cert</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>book now</t>
@@ -5406,13 +5362,11 @@
           <t>auto-enrolment</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>when staff hired</t>
@@ -5435,13 +5389,11 @@
           <t>PAYE/RTI filing</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>when staff hired</t>
@@ -5454,19 +5406,16 @@
           <t>UKAS body (future)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>ISO 27001</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>post-contract</t>
@@ -5479,19 +5428,16 @@
           <t>Insurer (future)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Cyber/PI</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>annual</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>get quotes</t>

</xml_diff>